<commit_message>
chore: complete append and merge
Next: learn M language
</commit_message>
<xml_diff>
--- a/6_Advanced_Data_Analysis/2_Data_Tables.xlsx
+++ b/6_Advanced_Data_Analysis/2_Data_Tables.xlsx
@@ -1,34 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27920"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Developer\_Courses\Excel\Excel_Data_Analytics_Course\6_Advanced_Data_Analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafli Ihsanuddin\Documents\GitHub\Data-Analyst\6_Advanced_Data_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF699739-AF38-4398-A5C0-59458B85094B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D37375E-5DB1-416E-A74D-5903A463D8E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="18336" windowHeight="10416" xr2:uid="{6C37AC85-509F-4D10-9DB1-F70D16D6FBAB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{6C37AC85-509F-4D10-9DB1-F70D16D6FBAB}"/>
   </bookViews>
   <sheets>
-    <sheet name="Original" sheetId="3" r:id="rId1"/>
-    <sheet name="Data_Table_One-Input" sheetId="1" r:id="rId2"/>
-    <sheet name="Data_Table_Two-Input" sheetId="2" r:id="rId3"/>
+    <sheet name="Two_Input" sheetId="4" r:id="rId1"/>
+    <sheet name="One_Input" sheetId="3" r:id="rId2"/>
+    <sheet name="Data_Table_One-Input" sheetId="1" r:id="rId3"/>
+    <sheet name="Data_Table_Two-Input" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="base" localSheetId="2">'Data_Table_Two-Input'!$C$3</definedName>
-    <definedName name="base" localSheetId="0">Original!$C$3</definedName>
+    <definedName name="base" localSheetId="3">'Data_Table_Two-Input'!$C$3</definedName>
+    <definedName name="base" localSheetId="1">One_Input!$C$3</definedName>
+    <definedName name="base" localSheetId="0">Two_Input!$C$3</definedName>
     <definedName name="base">'Data_Table_One-Input'!$C$3</definedName>
-    <definedName name="bonus" localSheetId="2">'Data_Table_Two-Input'!$C$4</definedName>
-    <definedName name="bonus" localSheetId="0">Original!$C$4</definedName>
+    <definedName name="bonus" localSheetId="3">'Data_Table_Two-Input'!$C$4</definedName>
+    <definedName name="bonus" localSheetId="1">One_Input!$C$4</definedName>
+    <definedName name="bonus" localSheetId="0">Two_Input!$C$4</definedName>
     <definedName name="bonus">'Data_Table_One-Input'!$C$4</definedName>
-    <definedName name="bonuys" localSheetId="2">'Data_Table_Two-Input'!$C$4</definedName>
-    <definedName name="bonuys" localSheetId="0">Original!$C$4</definedName>
+    <definedName name="bonuys" localSheetId="3">'Data_Table_Two-Input'!$C$4</definedName>
+    <definedName name="bonuys" localSheetId="1">One_Input!$C$4</definedName>
+    <definedName name="bonuys" localSheetId="0">Two_Input!$C$4</definedName>
     <definedName name="bonuys">'Data_Table_One-Input'!$C$4</definedName>
-    <definedName name="raise" localSheetId="2">'Data_Table_Two-Input'!$C$5</definedName>
-    <definedName name="raise" localSheetId="0">Original!$C$5</definedName>
+    <definedName name="raise" localSheetId="3">'Data_Table_Two-Input'!$C$5</definedName>
+    <definedName name="raise" localSheetId="1">One_Input!$C$5</definedName>
+    <definedName name="raise" localSheetId="0">Two_Input!$C$5</definedName>
     <definedName name="raise">'Data_Table_One-Input'!$C$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -43,8 +48,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -52,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="13">
   <si>
     <t>Base Salary</t>
   </si>
@@ -98,11 +101,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,6 +171,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1" tint="0.499984740745262"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -182,7 +199,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -428,24 +445,118 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -453,21 +564,29 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="17" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="7" fillId="2" borderId="17" xfId="3" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="18" xfId="3" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -480,14 +599,20 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="23" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="24" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="17" xfId="3" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="7" fillId="2" borderId="17" xfId="3" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="18" xfId="3" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -824,112 +949,203 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CAB43CA-5103-49AE-8216-4AB866E06AE4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F131963B-356E-4779-B30F-D9AF244FA5CC}">
   <dimension ref="B1:K14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="11.5234375" customWidth="1"/>
-    <col min="3" max="3" width="11.89453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="11" width="11.05078125" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" customWidth="1"/>
+    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="11" width="11.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6"/>
-    <row r="2" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B2" s="22" t="s">
+    <row r="1" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-    </row>
-    <row r="3" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="C2" s="29"/>
+      <c r="E2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="43" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="25">
         <v>100000</v>
       </c>
-      <c r="E3" s="11"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="21"/>
-    </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="E3" s="39">
+        <f>C14</f>
+        <v>566749.36181874992</v>
+      </c>
+      <c r="F3" s="40">
+        <v>0</v>
+      </c>
+      <c r="G3" s="41">
+        <v>0.05</v>
+      </c>
+      <c r="H3" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="I3" s="41">
+        <v>0.15</v>
+      </c>
+      <c r="J3" s="41">
+        <v>0.2</v>
+      </c>
+      <c r="K3" s="42">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="30">
+      <c r="C4" s="26">
         <v>0.1</v>
       </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="2"/>
-    </row>
-    <row r="5" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="E4" s="33">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="dataTable" ref="F4:K12" dt2D="1" dtr="1" r1="C4" r2="C5"/>
+        <v>500000</v>
+      </c>
+      <c r="G4" s="1">
+        <v>525000</v>
+      </c>
+      <c r="H4" s="1">
+        <v>550000.00000000012</v>
+      </c>
+      <c r="I4" s="1">
+        <v>574999.99999999988</v>
+      </c>
+      <c r="J4" s="1">
+        <v>600000</v>
+      </c>
+      <c r="K4" s="2">
+        <v>625000</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="27">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="E5" s="17"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="2"/>
-    </row>
-    <row r="6" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="E6" s="17"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="2"/>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="22" t="s">
+      <c r="E5" s="34">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="F5" s="1">
+        <v>505025.06256249989</v>
+      </c>
+      <c r="G5" s="1">
+        <v>530276.31569062488</v>
+      </c>
+      <c r="H5" s="1">
+        <v>555527.56881874998</v>
+      </c>
+      <c r="I5" s="1">
+        <v>580778.82194687473</v>
+      </c>
+      <c r="J5" s="1">
+        <v>606030.07507499983</v>
+      </c>
+      <c r="K5" s="2">
+        <v>631281.32820312493</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="E6" s="34">
+        <v>0.01</v>
+      </c>
+      <c r="F6" s="1">
+        <v>510100.50099999999</v>
+      </c>
+      <c r="G6" s="1">
+        <v>535605.52604999999</v>
+      </c>
+      <c r="H6" s="1">
+        <v>561110.55110000004</v>
+      </c>
+      <c r="I6" s="1">
+        <v>586615.57614999986</v>
+      </c>
+      <c r="J6" s="1">
+        <v>612120.60120000003</v>
+      </c>
+      <c r="K6" s="2">
+        <v>637625.62624999997</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B7" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="2"/>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="C7" s="29"/>
+      <c r="E7" s="34">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="F7" s="1">
+        <v>515226.6925624999</v>
+      </c>
+      <c r="G7" s="1">
+        <v>540988.02719062497</v>
+      </c>
+      <c r="H7" s="1">
+        <v>566749.36181874992</v>
+      </c>
+      <c r="I7" s="1">
+        <v>592510.69644687476</v>
+      </c>
+      <c r="J7" s="1">
+        <v>618272.03107499983</v>
+      </c>
+      <c r="K7" s="2">
+        <v>644033.3657031249</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B8" s="14" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="17"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="2"/>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="E8" s="34">
+        <v>0.02</v>
+      </c>
+      <c r="F8" s="1">
+        <v>520404.016</v>
+      </c>
+      <c r="G8" s="1">
+        <v>546424.21679999994</v>
+      </c>
+      <c r="H8" s="1">
+        <v>572444.41760000004</v>
+      </c>
+      <c r="I8" s="1">
+        <v>598464.61839999992</v>
+      </c>
+      <c r="J8" s="1">
+        <v>624484.81919999991</v>
+      </c>
+      <c r="K8" s="2">
+        <v>650505.02</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B9" s="9">
         <v>0</v>
       </c>
@@ -937,15 +1153,29 @@
         <f>(base*(1+raise)^B9)*(1+bonus)</f>
         <v>110000.00000000001</v>
       </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="E9" s="34">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="F9" s="1">
+        <v>525632.8515625</v>
+      </c>
+      <c r="G9" s="1">
+        <v>551914.494140625</v>
+      </c>
+      <c r="H9" s="1">
+        <v>578196.13671875</v>
+      </c>
+      <c r="I9" s="1">
+        <v>604477.77929687488</v>
+      </c>
+      <c r="J9" s="1">
+        <v>630759.42187499988</v>
+      </c>
+      <c r="K9" s="2">
+        <v>657041.064453125</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B10" s="9">
         <v>1</v>
       </c>
@@ -953,15 +1183,29 @@
         <f>(base*(1+raise)^B10)*(1+bonus)</f>
         <v>111650</v>
       </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="E10" s="34">
+        <v>0.03</v>
+      </c>
+      <c r="F10" s="1">
+        <v>530913.58100000001</v>
+      </c>
+      <c r="G10" s="1">
+        <v>557459.26005000004</v>
+      </c>
+      <c r="H10" s="1">
+        <v>584004.93910000008</v>
+      </c>
+      <c r="I10" s="1">
+        <v>610550.61814999988</v>
+      </c>
+      <c r="J10" s="1">
+        <v>637096.29719999991</v>
+      </c>
+      <c r="K10" s="2">
+        <v>663641.97625000007</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B11" s="9">
         <v>2</v>
       </c>
@@ -969,15 +1213,29 @@
         <f>(base*(1+raise)^B11)*(1+bonus)</f>
         <v>113324.74999999997</v>
       </c>
-      <c r="E11" s="17"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="2"/>
-    </row>
-    <row r="12" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="E11" s="34">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="F11" s="1">
+        <v>536246.58756249992</v>
+      </c>
+      <c r="G11" s="1">
+        <v>563058.91694062494</v>
+      </c>
+      <c r="H11" s="1">
+        <v>589871.24631874997</v>
+      </c>
+      <c r="I11" s="1">
+        <v>616683.57569687488</v>
+      </c>
+      <c r="J11" s="1">
+        <v>643495.9050749999</v>
+      </c>
+      <c r="K11" s="2">
+        <v>670308.23445312493</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="9">
         <v>3</v>
       </c>
@@ -985,15 +1243,29 @@
         <f>(base*(1+raise)^B12)*(1+bonus)</f>
         <v>115024.62124999997</v>
       </c>
-      <c r="E12" s="18"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="4"/>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+      <c r="E12" s="35">
+        <v>0.04</v>
+      </c>
+      <c r="F12" s="3">
+        <v>541632.25600000005</v>
+      </c>
+      <c r="G12" s="3">
+        <v>568713.86880000005</v>
+      </c>
+      <c r="H12" s="3">
+        <v>595795.48160000006</v>
+      </c>
+      <c r="I12" s="3">
+        <v>622877.09440000006</v>
+      </c>
+      <c r="J12" s="3">
+        <v>649958.70720000006</v>
+      </c>
+      <c r="K12" s="4">
+        <v>677040.32000000007</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B13" s="9">
         <v>4</v>
       </c>
@@ -1002,11 +1274,379 @@
         <v>116749.99056874996</v>
       </c>
     </row>
-    <row r="14" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="14" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B14" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="24">
+        <f>SUM(C9:C13)</f>
+        <v>566749.36181874992</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="F2:K2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F4:K12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color theme="3" tint="0.749992370372631"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CAB43CA-5103-49AE-8216-4AB866E06AE4}">
+  <dimension ref="B1:K14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="11.54296875" customWidth="1"/>
+    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="11" width="11.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="29"/>
+      <c r="E2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="25">
+        <v>100000</v>
+      </c>
+      <c r="E3" s="32"/>
+      <c r="F3" s="36">
+        <f>C9</f>
+        <v>110000.00000000001</v>
+      </c>
+      <c r="G3" s="37">
+        <f>C10</f>
+        <v>111650</v>
+      </c>
+      <c r="H3" s="37">
+        <f>C11</f>
+        <v>113324.74999999997</v>
+      </c>
+      <c r="I3" s="37">
+        <f>C12</f>
+        <v>115024.62124999997</v>
+      </c>
+      <c r="J3" s="37">
+        <f>C13</f>
+        <v>116749.99056874996</v>
+      </c>
+      <c r="K3" s="38">
+        <f>C14</f>
+        <v>566749.36181874992</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B4" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="26">
+        <v>0.1</v>
+      </c>
+      <c r="E4" s="33">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="dataTable" ref="F4:K12" dt2D="0" dtr="0" r1="C5"/>
+        <v>110000.00000000001</v>
+      </c>
+      <c r="G4" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="H4" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="I4" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="J4" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="K4" s="2">
+        <v>550000.00000000012</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="27">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="E5" s="34">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="F5" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="G5" s="1">
+        <v>110550</v>
+      </c>
+      <c r="H5" s="1">
+        <v>111102.74999999997</v>
+      </c>
+      <c r="I5" s="1">
+        <v>111658.26374999997</v>
+      </c>
+      <c r="J5" s="1">
+        <v>112216.55506874995</v>
+      </c>
+      <c r="K5" s="2">
+        <v>555527.56881874998</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="E6" s="34">
+        <v>0.01</v>
+      </c>
+      <c r="F6" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="G6" s="1">
+        <v>111100.00000000001</v>
+      </c>
+      <c r="H6" s="1">
+        <v>112211.00000000001</v>
+      </c>
+      <c r="I6" s="1">
+        <v>113333.11</v>
+      </c>
+      <c r="J6" s="1">
+        <v>114466.44110000001</v>
+      </c>
+      <c r="K6" s="2">
+        <v>561110.55110000004</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B7" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="29"/>
+      <c r="E7" s="34">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="F7" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="G7" s="1">
+        <v>111650</v>
+      </c>
+      <c r="H7" s="1">
+        <v>113324.74999999997</v>
+      </c>
+      <c r="I7" s="1">
+        <v>115024.62124999997</v>
+      </c>
+      <c r="J7" s="1">
+        <v>116749.99056874996</v>
+      </c>
+      <c r="K7" s="2">
+        <v>566749.36181874992</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="34">
+        <v>0.02</v>
+      </c>
+      <c r="F8" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="G8" s="1">
+        <v>112200.00000000001</v>
+      </c>
+      <c r="H8" s="1">
+        <v>114444.00000000001</v>
+      </c>
+      <c r="I8" s="1">
+        <v>116732.87999999999</v>
+      </c>
+      <c r="J8" s="1">
+        <v>119067.53760000001</v>
+      </c>
+      <c r="K8" s="2">
+        <v>572444.41760000004</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B9" s="9">
+        <v>0</v>
+      </c>
+      <c r="C9" s="7">
+        <f>(base*(1+raise)^B9)*(1+bonus)</f>
+        <v>110000.00000000001</v>
+      </c>
+      <c r="E9" s="34">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="F9" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="G9" s="1">
+        <v>112750</v>
+      </c>
+      <c r="H9" s="1">
+        <v>115568.75</v>
+      </c>
+      <c r="I9" s="1">
+        <v>118457.96875</v>
+      </c>
+      <c r="J9" s="1">
+        <v>121419.41796874997</v>
+      </c>
+      <c r="K9" s="2">
+        <v>578196.13671875</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B10" s="9">
+        <v>1</v>
+      </c>
+      <c r="C10" s="7">
+        <f>(base*(1+raise)^B10)*(1+bonus)</f>
+        <v>111650</v>
+      </c>
+      <c r="E10" s="34">
+        <v>0.03</v>
+      </c>
+      <c r="F10" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="G10" s="1">
+        <v>113300.00000000001</v>
+      </c>
+      <c r="H10" s="1">
+        <v>116699.00000000001</v>
+      </c>
+      <c r="I10" s="1">
+        <v>120199.97</v>
+      </c>
+      <c r="J10" s="1">
+        <v>123805.9691</v>
+      </c>
+      <c r="K10" s="2">
+        <v>584004.93910000008</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B11" s="9">
+        <v>2</v>
+      </c>
+      <c r="C11" s="7">
+        <f>(base*(1+raise)^B11)*(1+bonus)</f>
+        <v>113324.74999999997</v>
+      </c>
+      <c r="E11" s="34">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="F11" s="1">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="G11" s="1">
+        <v>113850</v>
+      </c>
+      <c r="H11" s="1">
+        <v>117834.75</v>
+      </c>
+      <c r="I11" s="1">
+        <v>121958.96624999998</v>
+      </c>
+      <c r="J11" s="1">
+        <v>126227.53006874998</v>
+      </c>
+      <c r="K11" s="2">
+        <v>589871.24631874997</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="9">
+        <v>3</v>
+      </c>
+      <c r="C12" s="7">
+        <f>(base*(1+raise)^B12)*(1+bonus)</f>
+        <v>115024.62124999997</v>
+      </c>
+      <c r="E12" s="35">
+        <v>0.04</v>
+      </c>
+      <c r="F12" s="3">
+        <v>110000.00000000001</v>
+      </c>
+      <c r="G12" s="3">
+        <v>114400.00000000001</v>
+      </c>
+      <c r="H12" s="3">
+        <v>118976.00000000003</v>
+      </c>
+      <c r="I12" s="3">
+        <v>123735.04000000002</v>
+      </c>
+      <c r="J12" s="3">
+        <v>128684.44160000002</v>
+      </c>
+      <c r="K12" s="4">
+        <v>595795.48160000006</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B13" s="9">
+        <v>4</v>
+      </c>
+      <c r="C13" s="7">
+        <f>(base*(1+raise)^B13)*(1+bonus)</f>
+        <v>116749.99056874996</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="24">
         <f>SUM(C9:C13)</f>
         <v>566749.36181874992</v>
       </c>
@@ -1016,57 +1656,78 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B7:C7"/>
   </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="F4:J12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color theme="3" tint="0.749992370372631"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4:K12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color theme="3" tint="0.749992370372631"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BC30AE1-3DCF-4D4C-A69F-2300F502F068}">
   <dimension ref="B1:K14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="11.5234375" customWidth="1"/>
-    <col min="3" max="3" width="11.89453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" customWidth="1"/>
+    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="11" width="11.05078125" customWidth="1"/>
+    <col min="6" max="11" width="11.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6"/>
-    <row r="2" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B2" s="22" t="s">
+    <row r="1" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="E2" s="26" t="s">
+      <c r="C2" s="29"/>
+      <c r="E2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="26" t="s">
+      <c r="F2" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="26" t="s">
+      <c r="G2" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="26" t="s">
+      <c r="H2" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="26" t="s">
+      <c r="I2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="26" t="s">
+      <c r="J2" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="26" t="s">
+      <c r="K2" s="22" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="3" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="25">
         <v>100000</v>
       </c>
-      <c r="E3" s="27"/>
+      <c r="E3" s="23"/>
       <c r="F3" s="12">
         <f>C9</f>
         <v>110000.00000000001</v>
@@ -1092,11 +1753,11 @@
         <v>566749.36181874992</v>
       </c>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="30">
+      <c r="C4" s="26">
         <v>0.1</v>
       </c>
       <c r="E4" s="17">
@@ -1122,11 +1783,11 @@
         <v>550000.00000000012</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="27">
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="E5" s="17">
@@ -1151,7 +1812,7 @@
         <v>555527.56881874998</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="6" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="E6" s="17">
         <v>0.01</v>
       </c>
@@ -1174,11 +1835,11 @@
         <v>561110.55110000004</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="22" t="s">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B7" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="23"/>
+      <c r="C7" s="29"/>
       <c r="E7" s="17">
         <v>1.4999999999999999E-2</v>
       </c>
@@ -1201,7 +1862,7 @@
         <v>566749.36181874992</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B8" s="14" t="s">
         <v>11</v>
       </c>
@@ -1230,7 +1891,7 @@
         <v>572444.41760000004</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B9" s="9">
         <v>0</v>
       </c>
@@ -1260,7 +1921,7 @@
         <v>578196.13671875</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B10" s="9">
         <v>1</v>
       </c>
@@ -1290,7 +1951,7 @@
         <v>584004.93910000008</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B11" s="9">
         <v>2</v>
       </c>
@@ -1320,7 +1981,7 @@
         <v>589871.24631874997</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="12" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="9">
         <v>3</v>
       </c>
@@ -1350,7 +2011,7 @@
         <v>595795.48160000006</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B13" s="9">
         <v>4</v>
       </c>
@@ -1359,11 +2020,11 @@
         <v>116749.99056874996</v>
       </c>
     </row>
-    <row r="14" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="14" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B14" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="24">
         <f>SUM(C9:C13)</f>
         <v>566749.36181874992</v>
       </c>
@@ -1406,41 +2067,41 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D225D585-7A9D-4201-AA98-B90D36B61978}">
   <dimension ref="B1:K14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="11.5234375" customWidth="1"/>
-    <col min="3" max="3" width="11.89453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" customWidth="1"/>
+    <col min="3" max="3" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="11" width="11.05078125" customWidth="1"/>
+    <col min="6" max="11" width="11.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6"/>
-    <row r="2" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B2" s="22" t="s">
+    <row r="1" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="23"/>
+      <c r="C2" s="29"/>
       <c r="E2" s="5"/>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-    </row>
-    <row r="3" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+    </row>
+    <row r="3" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="25">
         <v>100000</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="30" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="11">
@@ -1466,14 +2127,14 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="30">
+      <c r="C4" s="26">
         <v>0.1</v>
       </c>
-      <c r="D4" s="24"/>
+      <c r="D4" s="30"/>
       <c r="E4" s="16">
         <v>0</v>
       </c>
@@ -1497,14 +2158,14 @@
         <v>625000</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="27">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="D5" s="24"/>
+      <c r="D5" s="30"/>
       <c r="E5" s="17">
         <v>5.0000000000000001E-3</v>
       </c>
@@ -1527,8 +2188,8 @@
         <v>631281.32820312493</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="D6" s="24"/>
+    <row r="6" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D6" s="30"/>
       <c r="E6" s="17">
         <v>0.01</v>
       </c>
@@ -1551,12 +2212,12 @@
         <v>637625.62624999997</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="22" t="s">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B7" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="23"/>
-      <c r="D7" s="24"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="30"/>
       <c r="E7" s="17">
         <v>1.4999999999999999E-2</v>
       </c>
@@ -1579,14 +2240,14 @@
         <v>644033.3657031249</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B8" s="14" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="24"/>
+      <c r="D8" s="30"/>
       <c r="E8" s="17">
         <v>0.02</v>
       </c>
@@ -1609,7 +2270,7 @@
         <v>650505.02</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B9" s="9">
         <v>0</v>
       </c>
@@ -1617,7 +2278,7 @@
         <f>(base*(1+raise)^B9)*(1+bonus)</f>
         <v>110000.00000000001</v>
       </c>
-      <c r="D9" s="24"/>
+      <c r="D9" s="30"/>
       <c r="E9" s="17">
         <v>2.5000000000000001E-2</v>
       </c>
@@ -1640,7 +2301,7 @@
         <v>657041.064453125</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B10" s="9">
         <v>1</v>
       </c>
@@ -1648,7 +2309,7 @@
         <f>(base*(1+raise)^B10)*(1+bonus)</f>
         <v>111650</v>
       </c>
-      <c r="D10" s="24"/>
+      <c r="D10" s="30"/>
       <c r="E10" s="17">
         <v>0.03</v>
       </c>
@@ -1671,7 +2332,7 @@
         <v>663641.97625000007</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B11" s="9">
         <v>2</v>
       </c>
@@ -1679,7 +2340,7 @@
         <f>(base*(1+raise)^B11)*(1+bonus)</f>
         <v>113324.74999999997</v>
       </c>
-      <c r="D11" s="24"/>
+      <c r="D11" s="30"/>
       <c r="E11" s="17">
         <v>3.5000000000000003E-2</v>
       </c>
@@ -1702,7 +2363,7 @@
         <v>670308.23445312493</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="12" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="9">
         <v>3</v>
       </c>
@@ -1710,7 +2371,7 @@
         <f>(base*(1+raise)^B12)*(1+bonus)</f>
         <v>115024.62124999997</v>
       </c>
-      <c r="D12" s="24"/>
+      <c r="D12" s="30"/>
       <c r="E12" s="18">
         <v>0.04</v>
       </c>
@@ -1733,7 +2394,7 @@
         <v>677040.32000000007</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B13" s="9">
         <v>4</v>
       </c>
@@ -1742,11 +2403,11 @@
         <v>116749.99056874996</v>
       </c>
     </row>
-    <row r="14" spans="2:11" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="14" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B14" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="24">
         <f>SUM(C9:C13)</f>
         <v>566749.36181874992</v>
       </c>

</xml_diff>